<commit_message>
Adding ContactPage and MailPage to Github repository
</commit_message>
<xml_diff>
--- a/KeywordData/Keyword Data.xlsx
+++ b/KeywordData/Keyword Data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Appium\CI_CD_Jenkins_Git_Github\KeywordData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Appium\Git_Github_Jenkins_CI_CD\KeywordData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9FB24DD-4F81-4D98-9AF0-226A36289859}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{329881D6-9807-4D7C-AA1F-3008B4B2539E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{AEC07FBA-9F8E-4791-A519-104870105C04}"/>
+    <workbookView xWindow="3564" yWindow="1704" windowWidth="15624" windowHeight="8964" activeTab="1" xr2:uid="{AEC07FBA-9F8E-4791-A519-104870105C04}"/>
   </bookViews>
   <sheets>
     <sheet name="Mail" sheetId="3" r:id="rId1"/>

</xml_diff>

<commit_message>
Adding ContactTest, MailTest, ContactSearchEngine, MailSearchEngine and testng to Github repository
</commit_message>
<xml_diff>
--- a/KeywordData/Keyword Data.xlsx
+++ b/KeywordData/Keyword Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Appium\Git_Github_Jenkins_CI_CD\KeywordData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{329881D6-9807-4D7C-AA1F-3008B4B2539E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75F2F56B-ADEC-4E92-865B-5B52441290D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3564" yWindow="1704" windowWidth="15624" windowHeight="8964" activeTab="1" xr2:uid="{AEC07FBA-9F8E-4791-A519-104870105C04}"/>
+    <workbookView xWindow="3564" yWindow="1704" windowWidth="15624" windowHeight="8964" xr2:uid="{AEC07FBA-9F8E-4791-A519-104870105C04}"/>
   </bookViews>
   <sheets>
     <sheet name="Mail" sheetId="3" r:id="rId1"/>
@@ -542,17 +542,17 @@
     <col min="4" max="4" width="39.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:4" ht="18" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -753,6 +753,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Adding MyListener and Modified BaseClass and testng to Github repository
</commit_message>
<xml_diff>
--- a/KeywordData/Keyword Data.xlsx
+++ b/KeywordData/Keyword Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Appium\Git_Github_Jenkins_CI_CD\KeywordData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75F2F56B-ADEC-4E92-865B-5B52441290D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59DD09B0-DD0C-4029-982B-0CAA088BF1EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3564" yWindow="1704" windowWidth="15624" windowHeight="8964" xr2:uid="{AEC07FBA-9F8E-4791-A519-104870105C04}"/>
+    <workbookView xWindow="3564" yWindow="1704" windowWidth="15624" windowHeight="8964" activeTab="1" xr2:uid="{AEC07FBA-9F8E-4791-A519-104870105C04}"/>
   </bookViews>
   <sheets>
     <sheet name="Mail" sheetId="3" r:id="rId1"/>

</xml_diff>